<commit_message>
18 colleges' data done
</commit_message>
<xml_diff>
--- a/data/docs/proposed_schema (v3).xlsx
+++ b/data/docs/proposed_schema (v3).xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Farheen\DSE-Compass\data\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B92D3F9-16B0-4F0C-BC16-EED0AFCB2CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC59714F-E0BE-436C-8F8C-28A83BD5A8C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$E$104</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$E$105</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="120">
   <si>
     <t>1. college_details</t>
   </si>
@@ -379,6 +379,15 @@
   </si>
   <si>
     <t>AICTE approval status (Yes/No)</t>
+  </si>
+  <si>
+    <t>UNIQUE, NULL</t>
+  </si>
+  <si>
+    <t>admission_mode</t>
+  </si>
+  <si>
+    <t>CAP / University</t>
   </si>
 </sst>
 </file>
@@ -460,20 +469,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -754,7 +763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D111"/>
+  <dimension ref="A1:D112"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.44140625" customWidth="1"/>
@@ -764,12 +773,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -799,7 +808,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
@@ -807,7 +816,7 @@
         <v>35</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>38</v>
+        <v>117</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>39</v>
@@ -841,9 +850,9 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>6</v>
+        <v>118</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>40</v>
@@ -852,12 +861,12 @@
         <v>41</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>40</v>
@@ -866,12 +875,12 @@
         <v>41</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>40</v>
@@ -880,12 +889,12 @@
         <v>41</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>40</v>
@@ -894,54 +903,54 @@
         <v>41</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>41</v>
       </c>
       <c r="D11" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+    <row r="13" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="4" t="s">
+      <c r="B13" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+    <row r="14" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>11</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>48</v>
@@ -950,40 +959,40 @@
         <v>41</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+    <row r="16" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>13</v>
-      </c>
       <c r="B16" s="4" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>48</v>
@@ -992,146 +1001,146 @@
         <v>43</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D20" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B25" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
+    <row r="26" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C25" s="4" t="s">
+      <c r="B26" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D26" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
+    <row r="27" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C26" s="4" t="s">
+      <c r="B27" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D27" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
+    <row r="28" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C27" s="4" t="s">
+      <c r="B28" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C28" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D28" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
+    <row r="29" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
-        <v>111</v>
-      </c>
       <c r="B29" s="4" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>35</v>
@@ -1140,86 +1149,86 @@
         <v>43</v>
       </c>
       <c r="D30" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" s="4" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="7" t="s">
+      <c r="B35" s="11"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="3" t="s">
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B40" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C40" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D40" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="4" t="s">
+    <row r="41" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C40" s="4" t="s">
+      <c r="B41" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D40" s="4" t="s">
+      <c r="D41" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A41" s="4" t="s">
+    <row r="42" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A42" s="4" t="s">
         <v>1</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A42" s="4" t="s">
-        <v>17</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>35</v>
@@ -1228,156 +1237,156 @@
         <v>60</v>
       </c>
       <c r="D42" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A43" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D43" s="4" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A43" s="4" t="s">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B43" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="144" x14ac:dyDescent="0.3">
-      <c r="A44" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="B44" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>41</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>41</v>
       </c>
       <c r="D45" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D46" s="4" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="9" t="s">
+      <c r="A49" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="B49" s="9"/>
-      <c r="C49" s="9"/>
-      <c r="D49" s="9"/>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A52" s="7" t="s">
+      <c r="B50" s="11"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="11"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B52" s="7"/>
-      <c r="C52" s="7"/>
-      <c r="D52" s="7"/>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="3" t="s">
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B53" s="3" t="s">
+      <c r="B54" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C54" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D53" s="3" t="s">
+      <c r="D54" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="4" t="s">
+    <row r="55" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A55" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B54" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C54" s="4" t="s">
+      <c r="B55" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C55" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D54" s="4" t="s">
+      <c r="D55" s="4" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A55" s="4" t="s">
+    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C55" s="4" t="s">
+      <c r="B56" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C56" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D55" s="4" t="s">
+      <c r="D56" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A56" s="4" t="s">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B56" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C56" s="4" t="s">
+      <c r="B57" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C57" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D56" s="4" t="s">
+      <c r="D57" s="4" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A57" s="4" t="s">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D57" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>55</v>
@@ -1386,128 +1395,128 @@
         <v>43</v>
       </c>
       <c r="D58" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D59" s="4" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A60" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B60" s="8"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="8"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
       <c r="D61" s="6"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" s="9" t="s">
+      <c r="A62" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B62" s="7"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="7"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A63" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="B62" s="9"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="7" t="s">
+      <c r="B63" s="11"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="11"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A66" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B65" s="7"/>
-      <c r="C65" s="7"/>
-      <c r="D65" s="7"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="3" t="s">
+      <c r="B66" s="8"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="8"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="B67" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="C67" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D66" s="3" t="s">
+      <c r="D67" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A67" s="4" t="s">
+    <row r="68" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A68" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B67" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C67" s="4" t="s">
+      <c r="B68" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C68" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D67" s="4" t="s">
+      <c r="D68" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="4" t="s">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B68" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C68" s="4" t="s">
+      <c r="B69" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C69" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D68" s="4" t="s">
+      <c r="D69" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A69" s="4" t="s">
+    <row r="70" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A70" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B69" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C69" s="4" t="s">
+      <c r="B70" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C70" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D69" s="4" t="s">
+      <c r="D70" s="4" t="s">
         <v>92</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="B70" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C70" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>40</v>
@@ -1516,82 +1525,82 @@
         <v>41</v>
       </c>
       <c r="D72" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A73" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D73" s="4" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="1"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="1"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" s="7" t="s">
+      <c r="A75" s="1"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A76" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B75" s="7"/>
-      <c r="C75" s="7"/>
-      <c r="D75" s="7"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" s="3" t="s">
+      <c r="B76" s="8"/>
+      <c r="C76" s="8"/>
+      <c r="D76" s="8"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A77" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="B77" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C76" s="3" t="s">
+      <c r="C77" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D76" s="3" t="s">
+      <c r="D77" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A77" s="4" t="s">
+    <row r="78" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A78" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B77" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C77" s="4" t="s">
+      <c r="B78" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C78" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D77" s="4" t="s">
+      <c r="D78" s="4" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B78" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D78" s="4" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>22</v>
+        <v>110</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>43</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>99</v>
+        <v>22</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>40</v>
@@ -1600,14 +1609,22 @@
         <v>43</v>
       </c>
       <c r="D80" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D81" s="4" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" s="5"/>
-      <c r="B81" s="5"/>
-      <c r="C81" s="5"/>
-      <c r="D81" s="5"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="5"/>
@@ -1615,59 +1632,51 @@
       <c r="C82" s="5"/>
       <c r="D82" s="5"/>
     </row>
-    <row r="83" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="10" t="s">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" s="5"/>
+      <c r="B83" s="5"/>
+      <c r="C83" s="5"/>
+      <c r="D83" s="5"/>
+    </row>
+    <row r="84" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="B83" s="10"/>
-      <c r="C83" s="10"/>
-      <c r="D83" s="10"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A84" s="3" t="s">
+      <c r="B84" s="9"/>
+      <c r="C84" s="9"/>
+      <c r="D84" s="9"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B84" s="3" t="s">
+      <c r="B85" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C84" s="3" t="s">
+      <c r="C85" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D84" s="3" t="s">
+      <c r="D85" s="3" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A85" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B85" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C85" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
-        <v>17</v>
+        <v>82</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>35</v>
@@ -1676,101 +1685,101 @@
         <v>60</v>
       </c>
       <c r="D87" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A88" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D88" s="4" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" s="5"/>
-      <c r="B88" s="5"/>
-      <c r="C88" s="5"/>
-      <c r="D88" s="5"/>
-    </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="8" t="s">
+      <c r="A89" s="5"/>
+      <c r="B89" s="5"/>
+      <c r="C89" s="5"/>
+      <c r="D89" s="5"/>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A90" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B89" s="8"/>
-      <c r="C89" s="8"/>
-      <c r="D89" s="8"/>
-    </row>
-    <row r="90" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="11" t="s">
+      <c r="B90" s="6"/>
+      <c r="C90" s="6"/>
+      <c r="D90" s="6"/>
+    </row>
+    <row r="91" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="B90" s="11"/>
-      <c r="C90" s="11"/>
-      <c r="D90" s="11"/>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="9" t="s">
+      <c r="B91" s="10"/>
+      <c r="C91" s="10"/>
+      <c r="D91" s="10"/>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A92" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="B91" s="9"/>
-      <c r="C91" s="9"/>
-      <c r="D91" s="9"/>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A92" s="2"/>
-      <c r="B92" s="2"/>
-      <c r="C92" s="2"/>
-      <c r="D92" s="2"/>
+      <c r="B92" s="11"/>
+      <c r="C92" s="11"/>
+      <c r="D92" s="11"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" s="1"/>
+      <c r="A93" s="2"/>
+      <c r="B93" s="2"/>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" s="7" t="s">
+      <c r="A94" s="1"/>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A95" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="B94" s="7"/>
-      <c r="C94" s="7"/>
-      <c r="D94" s="7"/>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" s="3" t="s">
+      <c r="B95" s="8"/>
+      <c r="C95" s="8"/>
+      <c r="D95" s="8"/>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A96" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B95" s="3" t="s">
+      <c r="B96" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C95" s="3" t="s">
+      <c r="C96" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D95" s="3" t="s">
+      <c r="D96" s="3" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A96" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B96" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B97" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
-        <v>1</v>
+        <v>82</v>
       </c>
       <c r="B98" s="4" t="s">
         <v>35</v>
@@ -1779,27 +1788,38 @@
         <v>60</v>
       </c>
       <c r="D98" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A99" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D99" s="4" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A100" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B100" s="8"/>
-      <c r="C100" s="8"/>
-      <c r="D100" s="8"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" s="6" t="s">
-        <v>109</v>
+        <v>64</v>
       </c>
       <c r="B101" s="6"/>
       <c r="C101" s="6"/>
       <c r="D101" s="6"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A102" s="1"/>
+      <c r="A102" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B102" s="7"/>
+      <c r="C102" s="7"/>
+      <c r="D102" s="7"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" s="1"/>
@@ -1828,37 +1848,40 @@
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" s="1"/>
     </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A112" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A100:D100"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A35:D35"/>
     <mergeCell ref="A101:D101"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A65:D65"/>
-    <mergeCell ref="A75:D75"/>
-    <mergeCell ref="A94:D94"/>
-    <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A102:D102"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A66:D66"/>
+    <mergeCell ref="A76:D76"/>
+    <mergeCell ref="A95:D95"/>
+    <mergeCell ref="A84:D84"/>
+    <mergeCell ref="A91:D91"/>
     <mergeCell ref="A90:D90"/>
-    <mergeCell ref="A89:D89"/>
-    <mergeCell ref="A91:D91"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A92:D92"/>
+    <mergeCell ref="A63:D63"/>
     <mergeCell ref="A48:D48"/>
     <mergeCell ref="A49:D49"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A53:D53"/>
     <mergeCell ref="A61:D61"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A34:D34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="61" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
   <rowBreaks count="3" manualBreakCount="3">
-    <brk id="21" max="16383" man="1"/>
-    <brk id="50" max="4" man="1"/>
-    <brk id="63" max="4" man="1"/>
+    <brk id="22" max="16383" man="1"/>
+    <brk id="51" max="4" man="1"/>
+    <brk id="64" max="4" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
modified schema college_details, wrote its cleaning script
</commit_message>
<xml_diff>
--- a/data/docs/proposed_schema (v3).xlsx
+++ b/data/docs/proposed_schema (v3).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Farheen\DSE-Compass\data\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC59714F-E0BE-436C-8F8C-28A83BD5A8C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF6E59A-D1F2-48A1-B8EC-2845D7BF3B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$E$105</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$E$106</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="122">
   <si>
     <t>1. college_details</t>
   </si>
@@ -63,9 +63,6 @@
     <t>naac_grade</t>
   </si>
   <si>
-    <t>ugc_approved</t>
-  </si>
-  <si>
     <t>contact_no</t>
   </si>
   <si>
@@ -183,9 +180,6 @@
     <t>NAAC grade (e.g., A++, A+, A, B++)</t>
   </si>
   <si>
-    <t>UGC approval status (Yes/No)</t>
-  </si>
-  <si>
     <t>Official contact number</t>
   </si>
   <si>
@@ -198,9 +192,6 @@
     <t>REAL</t>
   </si>
   <si>
-    <t>Estimated total fees for entire degree program (3-4 years)</t>
-  </si>
-  <si>
     <t>Official college website URL</t>
   </si>
   <si>
@@ -384,17 +375,32 @@
     <t>UNIQUE, NULL</t>
   </si>
   <si>
-    <t>admission_mode</t>
-  </si>
-  <si>
-    <t>CAP / University</t>
+    <t>participates_in_cap</t>
+  </si>
+  <si>
+    <t>If college participates in CAP rounds (Yes/No)</t>
+  </si>
+  <si>
+    <t>ugc_recognized</t>
+  </si>
+  <si>
+    <t>UGC recognition status (Yes/No)</t>
+  </si>
+  <si>
+    <t>ugc_approved_section</t>
+  </si>
+  <si>
+    <t>Section under which UGC recognized the institute (sec 2(f) or sec 12(B))</t>
+  </si>
+  <si>
+    <t>Estimated total fees for entire degree program (3-4 years) (in Lakhs INR)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -414,6 +420,28 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -454,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -469,20 +497,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -763,7 +798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D112"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.44140625" customWidth="1"/>
@@ -773,25 +808,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -799,13 +834,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -813,13 +848,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -827,691 +862,691 @@
         <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>43</v>
-      </c>
       <c r="D6" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="D7" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="D10" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="D11" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="B17" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="4" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D17" s="4" t="s">
+    <row r="20" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="C20" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>57</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="C26" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D26" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="B27" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="D27" s="4" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B29" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>43</v>
-      </c>
       <c r="D29" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D32" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
+      <c r="A34" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
+      <c r="A35" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="12"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="12"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="C41" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="D41" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A41" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="B42" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C42" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C42" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="D42" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D43" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D47" s="4" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D44" s="4" t="s">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B49" s="13"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
+      <c r="B50" s="6"/>
+      <c r="C50" s="6"/>
+      <c r="D50" s="6"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B51" s="9"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B46" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="B49" s="7"/>
-      <c r="C49" s="7"/>
-      <c r="D49" s="7"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B50" s="11"/>
-      <c r="C50" s="11"/>
-      <c r="D50" s="11"/>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B53" s="8"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="8"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="3" t="s">
+      <c r="B54" s="12"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="12"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B55" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="C55" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="D55" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A55" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A57" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B56" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A57" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="B57" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B58" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A61" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B61" s="6"/>
-      <c r="C61" s="6"/>
-      <c r="D61" s="6"/>
+      <c r="B60" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="B62" s="7"/>
-      <c r="C62" s="7"/>
-      <c r="D62" s="7"/>
+      <c r="A62" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B62" s="13"/>
+      <c r="C62" s="13"/>
+      <c r="D62" s="13"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" s="11" t="s">
+      <c r="A63" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B63" s="6"/>
+      <c r="C63" s="6"/>
+      <c r="D63" s="6"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B64" s="9"/>
+      <c r="C64" s="9"/>
+      <c r="D64" s="9"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B67" s="14"/>
+      <c r="C67" s="14"/>
+      <c r="D67" s="14"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A68" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A69" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A70" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B63" s="11"/>
-      <c r="C63" s="11"/>
-      <c r="D63" s="11"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="8" t="s">
+      <c r="B70" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A71" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B66" s="8"/>
-      <c r="C66" s="8"/>
-      <c r="D66" s="8"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A68" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B68" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A69" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B69" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A70" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B70" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C70" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A71" s="4" t="s">
-        <v>88</v>
-      </c>
       <c r="B71" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
@@ -1519,118 +1554,126 @@
         <v>85</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B73" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C73" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C73" s="4" t="s">
-        <v>41</v>
-      </c>
       <c r="D73" s="4" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A74" s="1"/>
+      <c r="A74" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="1"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="B76" s="8"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
+      <c r="A76" s="1"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" s="3" t="s">
+      <c r="A77" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B77" s="7"/>
+      <c r="C77" s="7"/>
+      <c r="D77" s="7"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A78" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B78" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="C78" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C77" s="3" t="s">
+      <c r="D78" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D77" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A78" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B78" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D78" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="79" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>22</v>
+        <v>107</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" s="5"/>
-      <c r="B82" s="5"/>
-      <c r="C82" s="5"/>
-      <c r="D82" s="5"/>
+      <c r="A82" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="5"/>
@@ -1638,191 +1681,194 @@
       <c r="C83" s="5"/>
       <c r="D83" s="5"/>
     </row>
-    <row r="84" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="B84" s="9"/>
-      <c r="C84" s="9"/>
-      <c r="D84" s="9"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="3" t="s">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A84" s="5"/>
+      <c r="B84" s="5"/>
+      <c r="C84" s="5"/>
+      <c r="D84" s="5"/>
+    </row>
+    <row r="85" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B85" s="10"/>
+      <c r="C85" s="10"/>
+      <c r="D85" s="10"/>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A86" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B86" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B85" s="3" t="s">
+      <c r="C86" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C85" s="3" t="s">
+      <c r="D86" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="D85" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A86" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B86" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C86" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D86" s="4" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="B87" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C87" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C87" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="D87" s="4" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
-        <v>17</v>
+        <v>79</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="5"/>
-      <c r="B89" s="5"/>
-      <c r="C89" s="5"/>
-      <c r="D89" s="5"/>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A89" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B90" s="6"/>
-      <c r="C90" s="6"/>
-      <c r="D90" s="6"/>
-    </row>
-    <row r="91" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B91" s="10"/>
-      <c r="C91" s="10"/>
-      <c r="D91" s="10"/>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A90" s="5"/>
+      <c r="B90" s="5"/>
+      <c r="C90" s="5"/>
+      <c r="D90" s="5"/>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A91" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B91" s="8"/>
+      <c r="C91" s="8"/>
+      <c r="D91" s="8"/>
+    </row>
+    <row r="92" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="11" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B92" s="11"/>
       <c r="C92" s="11"/>
       <c r="D92" s="11"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" s="2"/>
-      <c r="B93" s="2"/>
-      <c r="C93" s="2"/>
-      <c r="D93" s="2"/>
+      <c r="A93" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B93" s="9"/>
+      <c r="C93" s="9"/>
+      <c r="D93" s="9"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" s="1"/>
+      <c r="A94" s="2"/>
+      <c r="B94" s="2"/>
+      <c r="C94" s="2"/>
+      <c r="D94" s="2"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="B95" s="8"/>
-      <c r="C95" s="8"/>
-      <c r="D95" s="8"/>
+      <c r="A95" s="1"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A96" s="3" t="s">
+      <c r="A96" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B96" s="7"/>
+      <c r="C96" s="7"/>
+      <c r="D96" s="7"/>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A97" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B97" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B96" s="3" t="s">
+      <c r="C97" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C96" s="3" t="s">
+      <c r="D97" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="D96" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A97" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B97" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C97" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D97" s="4" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B98" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C98" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C98" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="D98" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A100" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B99" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D99" s="4" t="s">
+      <c r="B100" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A102" s="8" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A101" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B101" s="6"/>
-      <c r="C101" s="6"/>
-      <c r="D101" s="6"/>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A102" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="B102" s="7"/>
-      <c r="C102" s="7"/>
-      <c r="D102" s="7"/>
+      <c r="B102" s="8"/>
+      <c r="C102" s="8"/>
+      <c r="D102" s="8"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A103" s="1"/>
+      <c r="A103" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B103" s="6"/>
+      <c r="C103" s="6"/>
+      <c r="D103" s="6"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" s="1"/>
@@ -1851,37 +1897,40 @@
     <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" s="1"/>
     </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A113" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A102:D102"/>
+    <mergeCell ref="A103:D103"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="A77:D77"/>
+    <mergeCell ref="A96:D96"/>
+    <mergeCell ref="A85:D85"/>
+    <mergeCell ref="A92:D92"/>
+    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="A93:D93"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A54:D54"/>
     <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A63:D63"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A25:D25"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A101:D101"/>
-    <mergeCell ref="A102:D102"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A66:D66"/>
-    <mergeCell ref="A76:D76"/>
-    <mergeCell ref="A95:D95"/>
-    <mergeCell ref="A84:D84"/>
-    <mergeCell ref="A91:D91"/>
-    <mergeCell ref="A90:D90"/>
-    <mergeCell ref="A92:D92"/>
-    <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="61" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
   <rowBreaks count="3" manualBreakCount="3">
-    <brk id="22" max="16383" man="1"/>
-    <brk id="51" max="4" man="1"/>
-    <brk id="64" max="4" man="1"/>
+    <brk id="23" max="16383" man="1"/>
+    <brk id="52" max="4" man="1"/>
+    <brk id="65" max="4" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finalized v3 of schema
</commit_message>
<xml_diff>
--- a/data/docs/proposed_schema (v3).xlsx
+++ b/data/docs/proposed_schema (v3).xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Farheen\DSE-Compass\data\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF6E59A-D1F2-48A1-B8EC-2845D7BF3B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CEDB6A7-74E4-4062-9EA1-71F7702B7867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$E$106</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$E$107</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="124">
   <si>
     <t>1. college_details</t>
   </si>
@@ -225,15 +225,6 @@
     <t>References branches.branch_id</t>
   </si>
   <si>
-    <t>Admission year (2025, 2024, 2023)</t>
-  </si>
-  <si>
-    <t>Admission category (GOPEN, LOPEN, GOBC, LOBC, GSC, LSC, GST, LST, GPWD)</t>
-  </si>
-  <si>
-    <t>Cutoff percentile for the specified category</t>
-  </si>
-  <si>
     <t>UNIQUE(college_id, branch_id, year, category)</t>
   </si>
   <si>
@@ -360,21 +351,12 @@
     <t>Approved intake capacity for branch (first year admission - FE)</t>
   </si>
   <si>
-    <t>latest_dse_intake</t>
-  </si>
-  <si>
-    <t>Approved intake capacity for branch (lateral entry - DSE)</t>
-  </si>
-  <si>
     <t>aicte_approved</t>
   </si>
   <si>
     <t>AICTE approval status (Yes/No)</t>
   </si>
   <si>
-    <t>UNIQUE, NULL</t>
-  </si>
-  <si>
     <t>participates_in_cap</t>
   </si>
   <si>
@@ -394,6 +376,42 @@
   </si>
   <si>
     <t>Estimated total fees for entire degree program (3-4 years) (in Lakhs INR)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">UNIQUE, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NULL</t>
+    </r>
+  </si>
+  <si>
+    <t>estimated_dse_intake</t>
+  </si>
+  <si>
+    <t>Estimated intake capacity for branch (lateral entry - DSE) (10% of FE rule)</t>
+  </si>
+  <si>
+    <t>dse_intake_2025</t>
+  </si>
+  <si>
+    <t>Intake of CAP 2025 (may include vacant seats of FE)</t>
+  </si>
+  <si>
+    <t>Admission category (GOPEN, LOPEN, GOBC, LOBC, GSC, LSC, GST, LST, GPWD, etc)</t>
+  </si>
+  <si>
+    <t>Cutoff percentile for the specified category for the specified year</t>
+  </si>
+  <si>
+    <t>Admission year (CAP 2025, 2024, 2023)</t>
   </si>
 </sst>
 </file>
@@ -434,13 +452,11 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -482,7 +498,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -497,27 +513,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -798,7 +815,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D114"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.44140625" customWidth="1"/>
@@ -808,12 +825,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -851,7 +868,7 @@
         <v>34</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>38</v>
@@ -882,21 +899,21 @@
         <v>40</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B7" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="6" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>116</v>
+      <c r="D7" s="14" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -985,7 +1002,7 @@
     </row>
     <row r="14" spans="1:4" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>47</v>
@@ -994,35 +1011,35 @@
         <v>40</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" s="6" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="14" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>120</v>
+      <c r="D16" s="14" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -1078,7 +1095,7 @@
         <v>42</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -1110,12 +1127,12 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
@@ -1187,111 +1204,111 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C31" s="4" t="s">
+    <row r="31" spans="1:4" s="6" customFormat="1" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C31" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="D31" s="4" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C32" s="4" t="s">
+      <c r="D31" s="14" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" s="6" customFormat="1" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="D32" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="13" t="s">
+      <c r="D32" s="14" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" s="6" customFormat="1" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B34" s="13"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="6" t="s">
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B40" s="12"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="12"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="3" t="s">
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B42" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C42" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D42" s="3" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A42" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>34</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>34</v>
@@ -1300,156 +1317,156 @@
         <v>57</v>
       </c>
       <c r="D44" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D45" s="4" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
+    <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B45" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="B46" s="4" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>40</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>40</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="13" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B49" s="13"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="13"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B50" s="6"/>
-      <c r="C50" s="6"/>
-      <c r="D50" s="6"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="15"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B51" s="9"/>
-      <c r="C51" s="9"/>
-      <c r="D51" s="9"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="12" t="s">
+      <c r="A51" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B52" s="13"/>
+      <c r="C52" s="13"/>
+      <c r="D52" s="13"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B54" s="12"/>
-      <c r="C54" s="12"/>
-      <c r="D54" s="12"/>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="3" t="s">
+      <c r="B55" s="9"/>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B56" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C56" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="D56" s="3" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A56" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B57" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C57" s="4" t="s">
+      <c r="B58" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C58" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D57" s="4" t="s">
+      <c r="D58" s="4" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A58" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B58" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>53</v>
@@ -1458,109 +1475,109 @@
         <v>42</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" s="13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A63" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="B62" s="13"/>
-      <c r="C62" s="13"/>
-      <c r="D62" s="13"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B63" s="6"/>
-      <c r="C63" s="6"/>
-      <c r="D63" s="6"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="15"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A64" s="9" t="s">
+      <c r="A64" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B64" s="8"/>
+      <c r="C64" s="8"/>
+      <c r="D64" s="8"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A65" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="B65" s="13"/>
+      <c r="C65" s="13"/>
+      <c r="D65" s="13"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A68" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B68" s="9"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="9"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A70" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A71" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="B67" s="14"/>
-      <c r="C67" s="14"/>
-      <c r="D67" s="14"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A69" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B69" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B70" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C70" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A71" s="4" t="s">
-        <v>81</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>39</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>39</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
@@ -1571,15 +1588,15 @@
         <v>39</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>39</v>
@@ -1588,82 +1605,82 @@
         <v>40</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" s="1"/>
+      <c r="A75" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="1"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B77" s="7"/>
-      <c r="C77" s="7"/>
-      <c r="D77" s="7"/>
+      <c r="A77" s="1"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" s="3" t="s">
+      <c r="A78" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B78" s="10"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="10"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B78" s="3" t="s">
+      <c r="B79" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C79" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D78" s="3" t="s">
+      <c r="D79" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A79" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B79" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>107</v>
+        <v>76</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>21</v>
+        <v>104</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>96</v>
+        <v>21</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>39</v>
@@ -1672,14 +1689,22 @@
         <v>42</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" s="5"/>
-      <c r="B83" s="5"/>
-      <c r="C83" s="5"/>
-      <c r="D83" s="5"/>
+      <c r="A83" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="5"/>
@@ -1687,59 +1712,51 @@
       <c r="C84" s="5"/>
       <c r="D84" s="5"/>
     </row>
-    <row r="85" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="B85" s="10"/>
-      <c r="C85" s="10"/>
-      <c r="D85" s="10"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" s="3" t="s">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" s="5"/>
+      <c r="B85" s="5"/>
+      <c r="C85" s="5"/>
+      <c r="D85" s="5"/>
+    </row>
+    <row r="86" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B86" s="11"/>
+      <c r="C86" s="11"/>
+      <c r="D86" s="11"/>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A87" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B86" s="3" t="s">
+      <c r="B87" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C86" s="3" t="s">
+      <c r="C87" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D86" s="3" t="s">
+      <c r="D87" s="3" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A87" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B87" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C87" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D87" s="4" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>34</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
-        <v>16</v>
+        <v>76</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>34</v>
@@ -1748,101 +1765,101 @@
         <v>57</v>
       </c>
       <c r="D89" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A90" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D90" s="4" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="5"/>
-      <c r="B90" s="5"/>
-      <c r="C90" s="5"/>
-      <c r="D90" s="5"/>
-    </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="8" t="s">
+      <c r="A91" s="5"/>
+      <c r="B91" s="5"/>
+      <c r="C91" s="5"/>
+      <c r="D91" s="5"/>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A92" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B91" s="8"/>
-      <c r="C91" s="8"/>
-      <c r="D91" s="8"/>
-    </row>
-    <row r="92" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="B92" s="11"/>
-      <c r="C92" s="11"/>
-      <c r="D92" s="11"/>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="B93" s="9"/>
-      <c r="C93" s="9"/>
-      <c r="D93" s="9"/>
+      <c r="B92" s="7"/>
+      <c r="C92" s="7"/>
+      <c r="D92" s="7"/>
+    </row>
+    <row r="93" spans="1:4" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B93" s="12"/>
+      <c r="C93" s="12"/>
+      <c r="D93" s="12"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" s="2"/>
-      <c r="B94" s="2"/>
-      <c r="C94" s="2"/>
-      <c r="D94" s="2"/>
+      <c r="A94" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B94" s="13"/>
+      <c r="C94" s="13"/>
+      <c r="D94" s="13"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" s="1"/>
+      <c r="A95" s="2"/>
+      <c r="B95" s="2"/>
+      <c r="C95" s="2"/>
+      <c r="D95" s="2"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A96" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B96" s="7"/>
-      <c r="C96" s="7"/>
-      <c r="D96" s="7"/>
+      <c r="A96" s="1"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A97" s="3" t="s">
+      <c r="A97" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="B97" s="10"/>
+      <c r="C97" s="10"/>
+      <c r="D97" s="10"/>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A98" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B97" s="3" t="s">
+      <c r="B98" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C97" s="3" t="s">
+      <c r="C98" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D97" s="3" t="s">
+      <c r="D98" s="3" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A98" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B98" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C98" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D98" s="4" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B99" s="4" t="s">
         <v>34</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="100" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
-        <v>1</v>
+        <v>76</v>
       </c>
       <c r="B100" s="4" t="s">
         <v>34</v>
@@ -1851,27 +1868,38 @@
         <v>57</v>
       </c>
       <c r="D100" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A101" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D101" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A102" s="8" t="s">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A103" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B102" s="8"/>
-      <c r="C102" s="8"/>
-      <c r="D102" s="8"/>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A103" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="B103" s="6"/>
-      <c r="C103" s="6"/>
-      <c r="D103" s="6"/>
+      <c r="B103" s="7"/>
+      <c r="C103" s="7"/>
+      <c r="D103" s="7"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A104" s="1"/>
+      <c r="A104" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B104" s="8"/>
+      <c r="C104" s="8"/>
+      <c r="D104" s="8"/>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" s="1"/>
@@ -1900,37 +1928,40 @@
     <row r="113" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A113" s="1"/>
     </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A114" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A102:D102"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A37:D37"/>
     <mergeCell ref="A103:D103"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A67:D67"/>
-    <mergeCell ref="A77:D77"/>
-    <mergeCell ref="A96:D96"/>
-    <mergeCell ref="A85:D85"/>
+    <mergeCell ref="A104:D104"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A68:D68"/>
+    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A86:D86"/>
+    <mergeCell ref="A93:D93"/>
     <mergeCell ref="A92:D92"/>
-    <mergeCell ref="A91:D91"/>
-    <mergeCell ref="A93:D93"/>
-    <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A94:D94"/>
+    <mergeCell ref="A65:D65"/>
     <mergeCell ref="A50:D50"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A55:D55"/>
     <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="61" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
   <rowBreaks count="3" manualBreakCount="3">
     <brk id="23" max="16383" man="1"/>
-    <brk id="52" max="4" man="1"/>
-    <brk id="65" max="4" man="1"/>
+    <brk id="53" max="4" man="1"/>
+    <brk id="66" max="4" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>